<commit_message>
Add bulk-import template download and test_date support
The bulk-import section had no way to grab a correctly-formatted file
to fill in, and its parser already supported a test_date column
(added in 7e4b553) that was never surfaced anywhere in the UI.

- Add a "Download Template" button that generates a header-only
  .xlsx with columns in the exact order the parser expects:
  participant_id, goniometer, ai_model, test_date, notes
- Clarify that multiple measurements for one participant are entered
  as multiple rows sharing the same participant_id, with no row limit
- Surface test_date in the template and the on-screen header guidance,
  completing the field the existing parser already read but the UI
  never mentioned
- Update the four extras/filesForTests fixtures (csv, json, xls, xlsx)
  to include test_date, keeping the same test scenarios: valid rows,
  a nonexistent-participant row that should be skipped, and a valid
  row after an error
</commit_message>
<xml_diff>
--- a/validata-app/extras/filesForTests/test_data.xlsx
+++ b/validata-app/extras/filesForTests/test_data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Measurements" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,6 +410,9 @@
         <v>ai_model</v>
       </c>
       <c r="D1" t="str">
+        <v>test_date</v>
+      </c>
+      <c r="E1" t="str">
         <v>notes</v>
       </c>
     </row>
@@ -424,6 +427,9 @@
         <v>44.9</v>
       </c>
       <c r="D2" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="E2" t="str">
         <v>Import Successful</v>
       </c>
     </row>
@@ -438,6 +444,9 @@
         <v>60.1</v>
       </c>
       <c r="D3" t="str">
+        <v>2026-06-12</v>
+      </c>
+      <c r="E3" t="str">
         <v>Another successful row</v>
       </c>
     </row>
@@ -452,6 +461,9 @@
         <v>90</v>
       </c>
       <c r="D4" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="E4" t="str">
         <v>This participant does not exist (should skip)</v>
       </c>
     </row>
@@ -466,12 +478,15 @@
         <v>31</v>
       </c>
       <c r="D5" t="str">
+        <v>2026-06-14</v>
+      </c>
+      <c r="E5" t="str">
         <v>Valid row after error</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>